<commit_message>
feat: verify live chart parity
</commit_message>
<xml_diff>
--- a/uiharness/fixtures/basic.xlsx
+++ b/uiharness/fixtures/basic.xlsx
@@ -98,84 +98,56 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Q1</c:v>
+            <c:strRef>
+              <c:f>Sheet1!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Q1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:tx>
           <c:cat>
-            <c:strLit>
-              <c:ptCount val="4"/>
-              <c:pt idx="0">
-                <c:v>North</c:v>
-              </c:pt>
-              <c:pt idx="1">
-                <c:v>South</c:v>
-              </c:pt>
-              <c:pt idx="2">
-                <c:v>East</c:v>
-              </c:pt>
-              <c:pt idx="3">
-                <c:v>West</c:v>
-              </c:pt>
-            </c:strLit>
+            <c:strRef>
+              <c:f>Sheet1!$A$2:$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>North</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>South</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>East</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>West</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
-            <c:numLit>
-              <c:formatCode>General</c:formatCode>
-              <c:ptCount val="4"/>
-              <c:pt idx="0">
-                <c:v>10</c:v>
-              </c:pt>
-              <c:pt idx="1">
-                <c:v>20</c:v>
-              </c:pt>
-              <c:pt idx="2">
-                <c:v>30</c:v>
-              </c:pt>
-              <c:pt idx="3">
-                <c:v>40</c:v>
-              </c:pt>
-            </c:numLit>
-          </c:val>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>Q2</c:v>
-          </c:tx>
-          <c:cat>
-            <c:strLit>
-              <c:ptCount val="4"/>
-              <c:pt idx="0">
-                <c:v>North</c:v>
-              </c:pt>
-              <c:pt idx="1">
-                <c:v>South</c:v>
-              </c:pt>
-              <c:pt idx="2">
-                <c:v>East</c:v>
-              </c:pt>
-              <c:pt idx="3">
-                <c:v>West</c:v>
-              </c:pt>
-            </c:strLit>
-          </c:cat>
-          <c:val>
-            <c:numLit>
-              <c:formatCode>General</c:formatCode>
-              <c:ptCount val="4"/>
-              <c:pt idx="0">
-                <c:v>14</c:v>
-              </c:pt>
-              <c:pt idx="1">
-                <c:v>24</c:v>
-              </c:pt>
-              <c:pt idx="2">
-                <c:v>34</c:v>
-              </c:pt>
-              <c:pt idx="3">
-                <c:v>44</c:v>
-              </c:pt>
-            </c:numLit>
+            <c:numRef>
+              <c:f>Sheet1!$B$2:$B$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>40</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
           </c:val>
         </c:ser>
         <c:axId val="111111111"/>

</xml_diff>